<commit_message>
Make sure code can run on computer and remove unnecessary GENuS imports
- makes sure main code runs on my computer (fixed missing folders, input files, wrong pointers)
- fixed global projection issues
- removed unnecessary GENuS imports
- TableS1_globa_inadequacies.xlsx Selenium value does not agree with calculations saved in CSV or how it is labeled on Fig1_intake_inadequacy_gdd_new.png
</commit_message>
<xml_diff>
--- a/tables/gdd_approach/TableS1_global_inadequacies.xlsx
+++ b/tables/gdd_approach/TableS1_global_inadequacies.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cfree/Dropbox/Chris/UCSB/projects/nutrition/global_intake_inadequacies/tables/gdd_approach/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://leidenuniv1-my.sharepoint.com/personal/haarsfter_vuw_leidenuniv_nl/Documents/Documents/global_intake_inadequacies/tables/gdd_approach/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5B1FC5-F03F-ED4B-ABD0-F1E9805CCB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{2B5B1FC5-F03F-ED4B-ABD0-F1E9805CCB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E27B8C7B-3DC0-4C47-8AA5-85ADF1F0A0BD}"/>
   <bookViews>
-    <workbookView xWindow="8200" yWindow="3020" windowWidth="27640" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TableS1_global_inadequacies" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -604,13 +617,17 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -967,24 +984,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E1" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F1" s="4"/>
     </row>
-    <row r="2" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -1003,8 +1020,10 @@
       <c r="F2" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+    </row>
+    <row r="3" spans="1:8" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1023,8 +1042,10 @@
       <c r="F3" s="3">
         <v>0.66878137468608001</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" s="3"/>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -1043,8 +1064,10 @@
       <c r="F4" s="3">
         <v>0.54509765630037799</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" s="3"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1063,8 +1086,10 @@
       <c r="F5" s="3">
         <v>0.53826293976609696</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5" s="3"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1083,8 +1108,10 @@
       <c r="F6" s="3">
         <v>0.53344068210470297</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G6" s="3"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -1103,8 +1130,10 @@
       <c r="F7" s="3">
         <v>0.51482228413961995</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7" s="3"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1123,8 +1152,10 @@
       <c r="F8" s="3">
         <v>0.47931646716159498</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G8" s="3"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -1143,8 +1174,10 @@
       <c r="F9" s="3">
         <v>0.39360560146255202</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9" s="3"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -1163,8 +1196,10 @@
       <c r="F10" s="3">
         <v>0.29727445433037802</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10" s="3"/>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1183,8 +1218,10 @@
       <c r="F11" s="3">
         <v>0.220751608012936</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G11" s="3"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1203,8 +1240,10 @@
       <c r="F12" s="3">
         <v>0.67542183240226605</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G12" s="3"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1223,28 +1262,32 @@
       <c r="F13" s="3">
         <v>0.66320568065459096</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="G13" s="3"/>
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="7">
         <v>4.8730244379302103</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="8">
         <v>0.64805168697545501</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G14" s="8"/>
+      <c r="H14" s="9"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1263,53 +1306,71 @@
       <c r="F15" s="3">
         <v>0.46153650032306198</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="G15" s="3"/>
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="7">
         <v>2.8296807901127599</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="8">
         <v>0.37631237704473802</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="G16" s="8"/>
+      <c r="H16" s="9"/>
+    </row>
+    <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="7">
         <v>2.3626996603556298</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="8">
         <v>0.31420969055516301</v>
       </c>
-    </row>
-    <row r="34" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="G17" s="8"/>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G18" s="3"/>
+    </row>
+    <row r="34" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E34" s="2"/>
       <c r="F34" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Classified as Internal | Intern</oddFooter>
+  </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{d465f887-04a9-4c17-8b62-103eddccf68b}" enabled="1" method="Standard" siteId="{ca2a7f76-dbd7-4ec0-9108-6b3d524fb7c8}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>